<commit_message>
add data from processing and ui for prompt
</commit_message>
<xml_diff>
--- a/tests/fixtures/LCA_Disclosure_Data_FY2099_Q1.xlsx
+++ b/tests/fixtures/LCA_Disclosure_Data_FY2099_Q1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LCA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCA" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,20 +469,30 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>NAICS_CODE</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>SECONDARY_ENTITY</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>WAGE_UNIT_OF_PAY</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>WORKSITE_CITY</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>PW_WAGE_LEVEL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>WAGE_RATE_OF_PAY_TO</t>
         </is>
@@ -536,25 +546,35 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Designer</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -578,7 +598,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Web and Digital Interface Designers</t>
+          <t>Video Game Designers</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -608,25 +628,35 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Designer</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -680,25 +710,35 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Graphic Designer</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Dallas</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -752,25 +792,35 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Designer</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Hour</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -824,25 +874,35 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Industrial Designer</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -893,21 +953,31 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Product Designer</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>519130</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Bi-Weekly</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -961,25 +1031,35 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Graphic Designer</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1033,25 +1113,35 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Graphic Designer</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1105,25 +1195,35 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Graphic Designer</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>Bi-Weekly</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1173,25 +1273,35 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Web Designer</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1251,20 +1361,30 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1323,20 +1443,30 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1395,20 +1525,30 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1467,20 +1607,30 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>95000</t>
         </is>
@@ -1539,20 +1689,30 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
+          <t>541430</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>95000</t>
         </is>

</xml_diff>